<commit_message>
Dodata su polja za mesto i adresu dobavljaca u bazu, kao i u tabelu Dobavljaci. Kroz eFakture se automatski preuzimaju i cuvaju ova dva polja.
</commit_message>
<xml_diff>
--- a/pomocna_knjiga_dobavljaca_excel.xlsx
+++ b/pomocna_knjiga_dobavljaca_excel.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="31">
-  <si>
-    <t>KNJIGA DOBAVLJAČA ZA PERIOD 01.01.2024. - 26.11.2024.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
+  <si>
+    <t>KNJIGA DOBAVLJAČA ZA PERIOD 01.01.2025. - 30.11.2025.</t>
   </si>
   <si>
     <t>Početno</t>
@@ -40,40 +40,49 @@
     <t>Potražuje</t>
   </si>
   <si>
-    <t>AMSS - CMV Beograd</t>
-  </si>
-  <si>
-    <t>CARDIOS - Novi Sad</t>
+    <t>Ada soft</t>
+  </si>
+  <si>
+    <t>Adeco doo</t>
+  </si>
+  <si>
+    <t>Agencija za bezbednost saobraćaja</t>
+  </si>
+  <si>
+    <t>Auto-moto savez Srbije</t>
+  </si>
+  <si>
+    <t>BC Group</t>
   </si>
   <si>
     <t>COOP SERVICE</t>
   </si>
   <si>
-    <t>DNEVNIK VOJVODINA PRES</t>
-  </si>
-  <si>
-    <t>FUTURA Novi Sad</t>
-  </si>
-  <si>
-    <t>GENERALI OSIGURANJE</t>
-  </si>
-  <si>
-    <t>GRADSKO ZELENILO</t>
+    <t>Generali osiguranje</t>
+  </si>
+  <si>
+    <t>HC-ING NOVI SAD</t>
+  </si>
+  <si>
+    <t>ING - PRO DOO BEOGRAD</t>
   </si>
   <si>
     <t xml:space="preserve">INTERSEC </t>
   </si>
   <si>
+    <t>IPC INFORM.POSLOVNI CENTAR</t>
+  </si>
+  <si>
     <t>JKP ČISTOĆA</t>
   </si>
   <si>
+    <t>JKP Gradsko zelenilo</t>
+  </si>
+  <si>
     <t>JKP INFORMATIKA</t>
   </si>
   <si>
-    <t>JP SLUŽBENI GLASNIK Beograd</t>
-  </si>
-  <si>
-    <t>Milosava Gelić - Novi Sad</t>
+    <t>JKP PARKING SERVIS NOVI SAD</t>
   </si>
   <si>
     <t>MS HERMES</t>
@@ -85,13 +94,19 @@
     <t>OFFICE TREND , Beograd</t>
   </si>
   <si>
+    <t>Poslovni biro doo</t>
+  </si>
+  <si>
     <t>PTT POŠTA</t>
   </si>
   <si>
-    <t>Suzana Ratković - Novi Sad</t>
-  </si>
-  <si>
-    <t>SZTR SOĆA SERVIS NOVI SAD</t>
+    <t>SAS-CS COMPANY - NOVI SAD</t>
+  </si>
+  <si>
+    <t>Srbolab</t>
+  </si>
+  <si>
+    <t>T&amp;M GROUP SOLUTIONS doo</t>
   </si>
   <si>
     <t>TDV FLEET SOLUTIONS</t>
@@ -101,9 +116,6 @@
   </si>
   <si>
     <t>UPRAVA ZA ZAJED.POSL.POKRAJ.ORGANA</t>
-  </si>
-  <si>
-    <t>ZANATSKA RADNJA BEG Novi Sad</t>
   </si>
   <si>
     <t>ZOMA</t>
@@ -462,15 +474,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="7" width="11" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
   </cols>
@@ -547,16 +557,16 @@
         <v>0</v>
       </c>
       <c r="D4" s="3">
-        <v>9400</v>
+        <v>516000.00</v>
       </c>
       <c r="E4" s="3">
-        <v>9400</v>
+        <v>516000.00</v>
       </c>
       <c r="F4" s="3">
-        <v>9400</v>
+        <v>516000.00</v>
       </c>
       <c r="G4" s="3">
-        <v>9400</v>
+        <v>516000.00</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
@@ -576,22 +586,22 @@
         <v>0</v>
       </c>
       <c r="D5" s="3">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="E5" s="3">
-        <v>200000</v>
+        <v>3456.00</v>
       </c>
       <c r="F5" s="3">
-        <v>200000</v>
+        <v>0</v>
       </c>
       <c r="G5" s="3">
-        <v>200000</v>
+        <v>3456.00</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>0</v>
+        <v>3456.00</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -602,19 +612,19 @@
         <v>0</v>
       </c>
       <c r="C6" s="3">
-        <v>98749.99000000001</v>
+        <v>0</v>
       </c>
       <c r="D6" s="3">
-        <v>1098733.99</v>
+        <v>3400.00</v>
       </c>
       <c r="E6" s="3">
-        <v>999984</v>
+        <v>3400.00</v>
       </c>
       <c r="F6" s="3">
-        <v>1098733.99</v>
+        <v>3400.00</v>
       </c>
       <c r="G6" s="3">
-        <v>1098733.99</v>
+        <v>3400.00</v>
       </c>
       <c r="H6" s="3">
         <v>0</v>
@@ -634,16 +644,16 @@
         <v>0</v>
       </c>
       <c r="D7" s="3">
-        <v>33868.8</v>
+        <v>28200.00</v>
       </c>
       <c r="E7" s="3">
-        <v>33868.8</v>
+        <v>28200.00</v>
       </c>
       <c r="F7" s="3">
-        <v>33868.8</v>
+        <v>28200.00</v>
       </c>
       <c r="G7" s="3">
-        <v>33868.8</v>
+        <v>28200.00</v>
       </c>
       <c r="H7" s="3">
         <v>0</v>
@@ -663,16 +673,16 @@
         <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>17304</v>
+        <v>49979.00</v>
       </c>
       <c r="E8" s="3">
-        <v>17304</v>
+        <v>49979.00</v>
       </c>
       <c r="F8" s="3">
-        <v>17304</v>
+        <v>49979.00</v>
       </c>
       <c r="G8" s="3">
-        <v>17304</v>
+        <v>49979.00</v>
       </c>
       <c r="H8" s="3">
         <v>0</v>
@@ -689,19 +699,19 @@
         <v>0</v>
       </c>
       <c r="C9" s="3">
-        <v>0</v>
+        <v>99998.40</v>
       </c>
       <c r="D9" s="3">
-        <v>57773.1</v>
+        <v>99998.40</v>
       </c>
       <c r="E9" s="3">
-        <v>57773.1</v>
+        <v>0</v>
       </c>
       <c r="F9" s="3">
-        <v>57773.1</v>
+        <v>99998.40</v>
       </c>
       <c r="G9" s="3">
-        <v>57773.1</v>
+        <v>99998.40</v>
       </c>
       <c r="H9" s="3">
         <v>0</v>
@@ -721,16 +731,16 @@
         <v>0</v>
       </c>
       <c r="D10" s="3">
-        <v>57600</v>
+        <v>52358.67</v>
       </c>
       <c r="E10" s="3">
-        <v>57600</v>
+        <v>52358.67</v>
       </c>
       <c r="F10" s="3">
-        <v>57600</v>
+        <v>52358.67</v>
       </c>
       <c r="G10" s="3">
-        <v>57600</v>
+        <v>52358.67</v>
       </c>
       <c r="H10" s="3">
         <v>0</v>
@@ -747,25 +757,25 @@
         <v>0</v>
       </c>
       <c r="C11" s="3">
-        <v>84223.57000000001</v>
+        <v>0</v>
       </c>
       <c r="D11" s="3">
-        <v>939008.05</v>
+        <v>136879.20</v>
       </c>
       <c r="E11" s="3">
-        <v>959918.4</v>
+        <v>136879.20</v>
       </c>
       <c r="F11" s="3">
-        <v>939008.05</v>
+        <v>136879.20</v>
       </c>
       <c r="G11" s="3">
-        <v>1044141.97</v>
+        <v>136879.20</v>
       </c>
       <c r="H11" s="3">
         <v>0</v>
       </c>
       <c r="I11" s="3">
-        <v>105133.92</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:9">
@@ -776,19 +786,19 @@
         <v>0</v>
       </c>
       <c r="C12" s="3">
-        <v>20307.06</v>
+        <v>0</v>
       </c>
       <c r="D12" s="3">
-        <v>227428.12</v>
+        <v>47300.00</v>
       </c>
       <c r="E12" s="3">
-        <v>207121.06</v>
+        <v>47300.00</v>
       </c>
       <c r="F12" s="3">
-        <v>227428.12</v>
+        <v>47300.00</v>
       </c>
       <c r="G12" s="3">
-        <v>227428.12</v>
+        <v>47300.00</v>
       </c>
       <c r="H12" s="3">
         <v>0</v>
@@ -805,25 +815,25 @@
         <v>0</v>
       </c>
       <c r="C13" s="3">
-        <v>1244</v>
+        <v>100562.88</v>
       </c>
       <c r="D13" s="3">
-        <v>13684</v>
+        <v>100562.88</v>
       </c>
       <c r="E13" s="3">
-        <v>13684</v>
+        <v>0</v>
       </c>
       <c r="F13" s="3">
-        <v>13684</v>
+        <v>100562.88</v>
       </c>
       <c r="G13" s="3">
-        <v>14928</v>
+        <v>100562.88</v>
       </c>
       <c r="H13" s="3">
         <v>0</v>
       </c>
       <c r="I13" s="3">
-        <v>1244</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:9">
@@ -837,16 +847,16 @@
         <v>0</v>
       </c>
       <c r="D14" s="3">
-        <v>47300</v>
+        <v>57000.00</v>
       </c>
       <c r="E14" s="3">
-        <v>47300</v>
+        <v>57000.00</v>
       </c>
       <c r="F14" s="3">
-        <v>47300</v>
+        <v>57000.00</v>
       </c>
       <c r="G14" s="3">
-        <v>47300</v>
+        <v>57000.00</v>
       </c>
       <c r="H14" s="3">
         <v>0</v>
@@ -863,19 +873,19 @@
         <v>0</v>
       </c>
       <c r="C15" s="3">
-        <v>0</v>
+        <v>22332.29</v>
       </c>
       <c r="D15" s="3">
-        <v>169526.5</v>
+        <v>245655.19</v>
       </c>
       <c r="E15" s="3">
-        <v>169526.5</v>
+        <v>223322.90</v>
       </c>
       <c r="F15" s="3">
-        <v>169526.5</v>
+        <v>245655.19</v>
       </c>
       <c r="G15" s="3">
-        <v>169526.5</v>
+        <v>245655.19</v>
       </c>
       <c r="H15" s="3">
         <v>0</v>
@@ -892,19 +902,19 @@
         <v>0</v>
       </c>
       <c r="C16" s="3">
-        <v>13209.04</v>
+        <v>0</v>
       </c>
       <c r="D16" s="3">
-        <v>128190.54</v>
+        <v>125400.00</v>
       </c>
       <c r="E16" s="3">
-        <v>114981.5</v>
+        <v>125400.00</v>
       </c>
       <c r="F16" s="3">
-        <v>128190.54</v>
+        <v>125400.00</v>
       </c>
       <c r="G16" s="3">
-        <v>128190.54</v>
+        <v>125400.00</v>
       </c>
       <c r="H16" s="3">
         <v>0</v>
@@ -921,19 +931,19 @@
         <v>0</v>
       </c>
       <c r="C17" s="3">
-        <v>0</v>
+        <v>1244.00</v>
       </c>
       <c r="D17" s="3">
-        <v>76048.8</v>
+        <v>13684.00</v>
       </c>
       <c r="E17" s="3">
-        <v>76048.8</v>
+        <v>12440.00</v>
       </c>
       <c r="F17" s="3">
-        <v>76048.8</v>
+        <v>13684.00</v>
       </c>
       <c r="G17" s="3">
-        <v>76048.8</v>
+        <v>13684.00</v>
       </c>
       <c r="H17" s="3">
         <v>0</v>
@@ -953,16 +963,16 @@
         <v>0</v>
       </c>
       <c r="D18" s="3">
-        <v>41947.2</v>
+        <v>266487.82</v>
       </c>
       <c r="E18" s="3">
-        <v>41947.2</v>
+        <v>266487.82</v>
       </c>
       <c r="F18" s="3">
-        <v>41947.2</v>
+        <v>266487.82</v>
       </c>
       <c r="G18" s="3">
-        <v>41947.2</v>
+        <v>266487.82</v>
       </c>
       <c r="H18" s="3">
         <v>0</v>
@@ -982,22 +992,22 @@
         <v>0</v>
       </c>
       <c r="D19" s="3">
-        <v>400000</v>
+        <v>124276.62</v>
       </c>
       <c r="E19" s="3">
-        <v>400000</v>
+        <v>169292.62</v>
       </c>
       <c r="F19" s="3">
-        <v>400000</v>
+        <v>124276.62</v>
       </c>
       <c r="G19" s="3">
-        <v>400000</v>
+        <v>169292.62</v>
       </c>
       <c r="H19" s="3">
         <v>0</v>
       </c>
       <c r="I19" s="3">
-        <v>0</v>
+        <v>45016.00</v>
       </c>
     </row>
     <row r="20" spans="1:9">
@@ -1011,16 +1021,16 @@
         <v>0</v>
       </c>
       <c r="D20" s="3">
-        <v>169526.5</v>
+        <v>189800.00</v>
       </c>
       <c r="E20" s="3">
-        <v>169526.5</v>
+        <v>189800.00</v>
       </c>
       <c r="F20" s="3">
-        <v>169526.5</v>
+        <v>189800.00</v>
       </c>
       <c r="G20" s="3">
-        <v>169526.5</v>
+        <v>189800.00</v>
       </c>
       <c r="H20" s="3">
         <v>0</v>
@@ -1040,22 +1050,22 @@
         <v>0</v>
       </c>
       <c r="D21" s="3">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3">
-        <v>1500</v>
+        <v>54028.80</v>
       </c>
       <c r="F21" s="3">
-        <v>1500</v>
+        <v>0</v>
       </c>
       <c r="G21" s="3">
-        <v>1500</v>
+        <v>54028.80</v>
       </c>
       <c r="H21" s="3">
         <v>0</v>
       </c>
       <c r="I21" s="3">
-        <v>0</v>
+        <v>54028.80</v>
       </c>
     </row>
     <row r="22" spans="1:9">
@@ -1066,19 +1076,19 @@
         <v>0</v>
       </c>
       <c r="C22" s="3">
-        <v>92820</v>
+        <v>0</v>
       </c>
       <c r="D22" s="3">
-        <v>1021020</v>
+        <v>4400.00</v>
       </c>
       <c r="E22" s="3">
-        <v>928200</v>
+        <v>4400.00</v>
       </c>
       <c r="F22" s="3">
-        <v>1021020</v>
+        <v>4400.00</v>
       </c>
       <c r="G22" s="3">
-        <v>1021020</v>
+        <v>4400.00</v>
       </c>
       <c r="H22" s="3">
         <v>0</v>
@@ -1095,25 +1105,25 @@
         <v>0</v>
       </c>
       <c r="C23" s="3">
-        <v>42388.76</v>
+        <v>0</v>
       </c>
       <c r="D23" s="3">
-        <v>449003.81</v>
+        <v>1500.00</v>
       </c>
       <c r="E23" s="3">
-        <v>412513.05</v>
+        <v>13500.00</v>
       </c>
       <c r="F23" s="3">
-        <v>449003.81</v>
+        <v>1500.00</v>
       </c>
       <c r="G23" s="3">
-        <v>454901.81</v>
+        <v>13500.00</v>
       </c>
       <c r="H23" s="3">
         <v>0</v>
       </c>
       <c r="I23" s="3">
-        <v>5898</v>
+        <v>12000.00</v>
       </c>
     </row>
     <row r="24" spans="1:9">
@@ -1124,25 +1134,25 @@
         <v>0</v>
       </c>
       <c r="C24" s="3">
-        <v>261483.82</v>
+        <v>0</v>
       </c>
       <c r="D24" s="3">
-        <v>890780.36</v>
+        <v>239160.00</v>
       </c>
       <c r="E24" s="3">
-        <v>674764.6</v>
+        <v>239160.00</v>
       </c>
       <c r="F24" s="3">
-        <v>890780.36</v>
+        <v>239160.00</v>
       </c>
       <c r="G24" s="3">
-        <v>936248.42</v>
+        <v>239160.00</v>
       </c>
       <c r="H24" s="3">
         <v>0</v>
       </c>
       <c r="I24" s="3">
-        <v>45468.06</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:9">
@@ -1153,19 +1163,19 @@
         <v>0</v>
       </c>
       <c r="C25" s="3">
-        <v>4500</v>
+        <v>0</v>
       </c>
       <c r="D25" s="3">
-        <v>4500</v>
+        <v>10000.00</v>
       </c>
       <c r="E25" s="3">
-        <v>0</v>
+        <v>10000.00</v>
       </c>
       <c r="F25" s="3">
-        <v>4500</v>
+        <v>10000.00</v>
       </c>
       <c r="G25" s="3">
-        <v>4500</v>
+        <v>10000.00</v>
       </c>
       <c r="H25" s="3">
         <v>0</v>
@@ -1185,22 +1195,138 @@
         <v>0</v>
       </c>
       <c r="D26" s="3">
-        <v>441894</v>
+        <v>3669105.60</v>
       </c>
       <c r="E26" s="3">
-        <v>441894</v>
+        <v>3882225.60</v>
       </c>
       <c r="F26" s="3">
-        <v>441894</v>
+        <v>3669105.60</v>
       </c>
       <c r="G26" s="3">
-        <v>441894</v>
+        <v>3882225.60</v>
       </c>
       <c r="H26" s="3">
         <v>0</v>
       </c>
       <c r="I26" s="3">
-        <v>0</v>
+        <v>213120.00</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="3">
+        <v>0</v>
+      </c>
+      <c r="C27" s="3">
+        <v>92820.00</v>
+      </c>
+      <c r="D27" s="3">
+        <v>1021020.00</v>
+      </c>
+      <c r="E27" s="3">
+        <v>928200.00</v>
+      </c>
+      <c r="F27" s="3">
+        <v>1021020.00</v>
+      </c>
+      <c r="G27" s="3">
+        <v>1021020.00</v>
+      </c>
+      <c r="H27" s="3">
+        <v>0</v>
+      </c>
+      <c r="I27" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>32</v>
+      </c>
+      <c r="B28" s="3">
+        <v>0</v>
+      </c>
+      <c r="C28" s="3">
+        <v>48064.79</v>
+      </c>
+      <c r="D28" s="3">
+        <v>524886.87</v>
+      </c>
+      <c r="E28" s="3">
+        <v>476822.08</v>
+      </c>
+      <c r="F28" s="3">
+        <v>524886.87</v>
+      </c>
+      <c r="G28" s="3">
+        <v>524886.87</v>
+      </c>
+      <c r="H28" s="3">
+        <v>0</v>
+      </c>
+      <c r="I28" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="3">
+        <v>0</v>
+      </c>
+      <c r="C29" s="3">
+        <v>319490.27</v>
+      </c>
+      <c r="D29" s="3">
+        <v>1202130.75</v>
+      </c>
+      <c r="E29" s="3">
+        <v>974675.06</v>
+      </c>
+      <c r="F29" s="3">
+        <v>1202130.75</v>
+      </c>
+      <c r="G29" s="3">
+        <v>1294165.33</v>
+      </c>
+      <c r="H29" s="3">
+        <v>0</v>
+      </c>
+      <c r="I29" s="3">
+        <v>92034.58</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" t="s">
+        <v>34</v>
+      </c>
+      <c r="B30" s="3">
+        <v>0</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0</v>
+      </c>
+      <c r="D30" s="3">
+        <v>503982.00</v>
+      </c>
+      <c r="E30" s="3">
+        <v>536562.00</v>
+      </c>
+      <c r="F30" s="3">
+        <v>503982.00</v>
+      </c>
+      <c r="G30" s="3">
+        <v>536562.00</v>
+      </c>
+      <c r="H30" s="3">
+        <v>0</v>
+      </c>
+      <c r="I30" s="3">
+        <v>32580.00</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ispravljena greska kod stampe IOS
</commit_message>
<xml_diff>
--- a/pomocna_knjiga_dobavljaca_excel.xlsx
+++ b/pomocna_knjiga_dobavljaca_excel.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="35">
-  <si>
-    <t>KNJIGA DOBAVLJAČA ZA PERIOD 01.01.2025. - 30.11.2025.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
+  <si>
+    <t>KNJIGA DOBAVLJAČA ZA PERIOD 07.10.2025. - 26.12.2025.</t>
   </si>
   <si>
     <t>Početno</t>
@@ -40,55 +40,25 @@
     <t>Potražuje</t>
   </si>
   <si>
-    <t>Ada soft</t>
-  </si>
-  <si>
     <t>Adeco doo</t>
   </si>
   <si>
-    <t>Agencija za bezbednost saobraćaja</t>
-  </si>
-  <si>
     <t>Auto-moto savez Srbije</t>
   </si>
   <si>
-    <t>BC Group</t>
-  </si>
-  <si>
-    <t>COOP SERVICE</t>
-  </si>
-  <si>
-    <t>Generali osiguranje</t>
-  </si>
-  <si>
-    <t>HC-ING NOVI SAD</t>
-  </si>
-  <si>
     <t>ING - PRO DOO BEOGRAD</t>
   </si>
   <si>
-    <t xml:space="preserve">INTERSEC </t>
-  </si>
-  <si>
-    <t>IPC INFORM.POSLOVNI CENTAR</t>
-  </si>
-  <si>
     <t>JKP ČISTOĆA</t>
   </si>
   <si>
     <t>JKP Gradsko zelenilo</t>
   </si>
   <si>
-    <t>JKP INFORMATIKA</t>
-  </si>
-  <si>
-    <t>JKP PARKING SERVIS NOVI SAD</t>
-  </si>
-  <si>
-    <t>MS HERMES</t>
-  </si>
-  <si>
-    <t>NIS GASPROM</t>
+    <t>JKP Informatika</t>
+  </si>
+  <si>
+    <t>M-S Hermes</t>
   </si>
   <si>
     <t>OFFICE TREND , Beograd</t>
@@ -101,9 +71,6 @@
   </si>
   <si>
     <t>SAS-CS COMPANY - NOVI SAD</t>
-  </si>
-  <si>
-    <t>Srbolab</t>
   </si>
   <si>
     <t>T&amp;M GROUP SOLUTIONS doo</t>
@@ -474,15 +441,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10" bestFit="1" customWidth="1"/>
-    <col min="4" max="7" width="11" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -557,16 +523,16 @@
         <v>0</v>
       </c>
       <c r="D4" s="3">
-        <v>516000.00</v>
+        <v>3456.00</v>
       </c>
       <c r="E4" s="3">
-        <v>516000.00</v>
+        <v>3456.00</v>
       </c>
       <c r="F4" s="3">
-        <v>516000.00</v>
+        <v>3456.00</v>
       </c>
       <c r="G4" s="3">
-        <v>516000.00</v>
+        <v>3456.00</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
@@ -586,22 +552,22 @@
         <v>0</v>
       </c>
       <c r="D5" s="3">
-        <v>0</v>
+        <v>28200.00</v>
       </c>
       <c r="E5" s="3">
-        <v>3456.00</v>
+        <v>28200.00</v>
       </c>
       <c r="F5" s="3">
-        <v>0</v>
+        <v>28200.00</v>
       </c>
       <c r="G5" s="3">
-        <v>3456.00</v>
+        <v>28200.00</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
       </c>
       <c r="I5" s="3">
-        <v>3456.00</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -615,16 +581,16 @@
         <v>0</v>
       </c>
       <c r="D6" s="3">
-        <v>3400.00</v>
+        <v>47300.00</v>
       </c>
       <c r="E6" s="3">
-        <v>3400.00</v>
+        <v>47300.00</v>
       </c>
       <c r="F6" s="3">
-        <v>3400.00</v>
+        <v>47300.00</v>
       </c>
       <c r="G6" s="3">
-        <v>3400.00</v>
+        <v>47300.00</v>
       </c>
       <c r="H6" s="3">
         <v>0</v>
@@ -644,22 +610,22 @@
         <v>0</v>
       </c>
       <c r="D7" s="3">
-        <v>28200.00</v>
+        <v>22332.29</v>
       </c>
       <c r="E7" s="3">
-        <v>28200.00</v>
+        <v>44664.58</v>
       </c>
       <c r="F7" s="3">
-        <v>28200.00</v>
+        <v>22332.29</v>
       </c>
       <c r="G7" s="3">
-        <v>28200.00</v>
+        <v>44664.58</v>
       </c>
       <c r="H7" s="3">
         <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>0</v>
+        <v>22332.29</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -673,16 +639,16 @@
         <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>49979.00</v>
+        <v>75600.00</v>
       </c>
       <c r="E8" s="3">
-        <v>49979.00</v>
+        <v>75600.00</v>
       </c>
       <c r="F8" s="3">
-        <v>49979.00</v>
+        <v>75600.00</v>
       </c>
       <c r="G8" s="3">
-        <v>49979.00</v>
+        <v>75600.00</v>
       </c>
       <c r="H8" s="3">
         <v>0</v>
@@ -699,25 +665,25 @@
         <v>0</v>
       </c>
       <c r="C9" s="3">
-        <v>99998.40</v>
+        <v>0</v>
       </c>
       <c r="D9" s="3">
-        <v>99998.40</v>
+        <v>2488.00</v>
       </c>
       <c r="E9" s="3">
-        <v>0</v>
+        <v>3732.00</v>
       </c>
       <c r="F9" s="3">
-        <v>99998.40</v>
+        <v>2488.00</v>
       </c>
       <c r="G9" s="3">
-        <v>99998.40</v>
+        <v>3732.00</v>
       </c>
       <c r="H9" s="3">
         <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>0</v>
+        <v>1244.00</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -731,16 +697,16 @@
         <v>0</v>
       </c>
       <c r="D10" s="3">
-        <v>52358.67</v>
+        <v>87463.80</v>
       </c>
       <c r="E10" s="3">
-        <v>52358.67</v>
+        <v>87463.80</v>
       </c>
       <c r="F10" s="3">
-        <v>52358.67</v>
+        <v>87463.80</v>
       </c>
       <c r="G10" s="3">
-        <v>52358.67</v>
+        <v>87463.80</v>
       </c>
       <c r="H10" s="3">
         <v>0</v>
@@ -760,16 +726,16 @@
         <v>0</v>
       </c>
       <c r="D11" s="3">
-        <v>136879.20</v>
+        <v>54028.80</v>
       </c>
       <c r="E11" s="3">
-        <v>136879.20</v>
+        <v>54028.80</v>
       </c>
       <c r="F11" s="3">
-        <v>136879.20</v>
+        <v>54028.80</v>
       </c>
       <c r="G11" s="3">
-        <v>136879.20</v>
+        <v>54028.80</v>
       </c>
       <c r="H11" s="3">
         <v>0</v>
@@ -789,16 +755,16 @@
         <v>0</v>
       </c>
       <c r="D12" s="3">
-        <v>47300.00</v>
+        <v>4400.00</v>
       </c>
       <c r="E12" s="3">
-        <v>47300.00</v>
+        <v>4400.00</v>
       </c>
       <c r="F12" s="3">
-        <v>47300.00</v>
+        <v>4400.00</v>
       </c>
       <c r="G12" s="3">
-        <v>47300.00</v>
+        <v>4400.00</v>
       </c>
       <c r="H12" s="3">
         <v>0</v>
@@ -815,19 +781,19 @@
         <v>0</v>
       </c>
       <c r="C13" s="3">
-        <v>100562.88</v>
+        <v>0</v>
       </c>
       <c r="D13" s="3">
-        <v>100562.88</v>
+        <v>12000.00</v>
       </c>
       <c r="E13" s="3">
-        <v>0</v>
+        <v>12000.00</v>
       </c>
       <c r="F13" s="3">
-        <v>100562.88</v>
+        <v>12000.00</v>
       </c>
       <c r="G13" s="3">
-        <v>100562.88</v>
+        <v>12000.00</v>
       </c>
       <c r="H13" s="3">
         <v>0</v>
@@ -847,16 +813,16 @@
         <v>0</v>
       </c>
       <c r="D14" s="3">
-        <v>57000.00</v>
+        <v>239160.00</v>
       </c>
       <c r="E14" s="3">
-        <v>57000.00</v>
+        <v>239160.00</v>
       </c>
       <c r="F14" s="3">
-        <v>57000.00</v>
+        <v>239160.00</v>
       </c>
       <c r="G14" s="3">
-        <v>57000.00</v>
+        <v>239160.00</v>
       </c>
       <c r="H14" s="3">
         <v>0</v>
@@ -873,22 +839,22 @@
         <v>0</v>
       </c>
       <c r="C15" s="3">
-        <v>22332.29</v>
+        <v>0</v>
       </c>
       <c r="D15" s="3">
-        <v>245655.19</v>
+        <v>970488.00</v>
       </c>
       <c r="E15" s="3">
-        <v>223322.90</v>
+        <v>902696.40</v>
       </c>
       <c r="F15" s="3">
-        <v>245655.19</v>
+        <v>970488.00</v>
       </c>
       <c r="G15" s="3">
-        <v>245655.19</v>
+        <v>902696.40</v>
       </c>
       <c r="H15" s="3">
-        <v>0</v>
+        <v>67791.60</v>
       </c>
       <c r="I15" s="3">
         <v>0</v>
@@ -905,22 +871,22 @@
         <v>0</v>
       </c>
       <c r="D16" s="3">
-        <v>125400.00</v>
+        <v>173663.22</v>
       </c>
       <c r="E16" s="3">
-        <v>125400.00</v>
+        <v>266483.22</v>
       </c>
       <c r="F16" s="3">
-        <v>125400.00</v>
+        <v>173663.22</v>
       </c>
       <c r="G16" s="3">
-        <v>125400.00</v>
+        <v>266483.22</v>
       </c>
       <c r="H16" s="3">
         <v>0</v>
       </c>
       <c r="I16" s="3">
-        <v>0</v>
+        <v>92820.00</v>
       </c>
     </row>
     <row r="17" spans="1:9">
@@ -931,25 +897,25 @@
         <v>0</v>
       </c>
       <c r="C17" s="3">
-        <v>1244.00</v>
+        <v>0</v>
       </c>
       <c r="D17" s="3">
-        <v>13684.00</v>
+        <v>95748.29</v>
       </c>
       <c r="E17" s="3">
-        <v>12440.00</v>
+        <v>143932.09</v>
       </c>
       <c r="F17" s="3">
-        <v>13684.00</v>
+        <v>95748.29</v>
       </c>
       <c r="G17" s="3">
-        <v>13684.00</v>
+        <v>143932.09</v>
       </c>
       <c r="H17" s="3">
         <v>0</v>
       </c>
       <c r="I17" s="3">
-        <v>0</v>
+        <v>48183.80</v>
       </c>
     </row>
     <row r="18" spans="1:9">
@@ -963,19 +929,19 @@
         <v>0</v>
       </c>
       <c r="D18" s="3">
-        <v>266487.82</v>
+        <v>358355.02</v>
       </c>
       <c r="E18" s="3">
-        <v>266487.82</v>
+        <v>183325.26</v>
       </c>
       <c r="F18" s="3">
-        <v>266487.82</v>
+        <v>358355.02</v>
       </c>
       <c r="G18" s="3">
-        <v>266487.82</v>
+        <v>183325.26</v>
       </c>
       <c r="H18" s="3">
-        <v>0</v>
+        <v>175029.76</v>
       </c>
       <c r="I18" s="3">
         <v>0</v>
@@ -992,341 +958,22 @@
         <v>0</v>
       </c>
       <c r="D19" s="3">
-        <v>124276.62</v>
+        <v>244080.00</v>
       </c>
       <c r="E19" s="3">
-        <v>169292.62</v>
+        <v>244080.00</v>
       </c>
       <c r="F19" s="3">
-        <v>124276.62</v>
+        <v>244080.00</v>
       </c>
       <c r="G19" s="3">
-        <v>169292.62</v>
+        <v>244080.00</v>
       </c>
       <c r="H19" s="3">
         <v>0</v>
       </c>
       <c r="I19" s="3">
-        <v>45016.00</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" t="s">
-        <v>24</v>
-      </c>
-      <c r="B20" s="3">
-        <v>0</v>
-      </c>
-      <c r="C20" s="3">
-        <v>0</v>
-      </c>
-      <c r="D20" s="3">
-        <v>189800.00</v>
-      </c>
-      <c r="E20" s="3">
-        <v>189800.00</v>
-      </c>
-      <c r="F20" s="3">
-        <v>189800.00</v>
-      </c>
-      <c r="G20" s="3">
-        <v>189800.00</v>
-      </c>
-      <c r="H20" s="3">
-        <v>0</v>
-      </c>
-      <c r="I20" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" t="s">
-        <v>25</v>
-      </c>
-      <c r="B21" s="3">
-        <v>0</v>
-      </c>
-      <c r="C21" s="3">
-        <v>0</v>
-      </c>
-      <c r="D21" s="3">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3">
-        <v>54028.80</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3">
-        <v>54028.80</v>
-      </c>
-      <c r="H21" s="3">
-        <v>0</v>
-      </c>
-      <c r="I21" s="3">
-        <v>54028.80</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" t="s">
-        <v>26</v>
-      </c>
-      <c r="B22" s="3">
-        <v>0</v>
-      </c>
-      <c r="C22" s="3">
-        <v>0</v>
-      </c>
-      <c r="D22" s="3">
-        <v>4400.00</v>
-      </c>
-      <c r="E22" s="3">
-        <v>4400.00</v>
-      </c>
-      <c r="F22" s="3">
-        <v>4400.00</v>
-      </c>
-      <c r="G22" s="3">
-        <v>4400.00</v>
-      </c>
-      <c r="H22" s="3">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="3">
-        <v>0</v>
-      </c>
-      <c r="C23" s="3">
-        <v>0</v>
-      </c>
-      <c r="D23" s="3">
-        <v>1500.00</v>
-      </c>
-      <c r="E23" s="3">
-        <v>13500.00</v>
-      </c>
-      <c r="F23" s="3">
-        <v>1500.00</v>
-      </c>
-      <c r="G23" s="3">
-        <v>13500.00</v>
-      </c>
-      <c r="H23" s="3">
-        <v>0</v>
-      </c>
-      <c r="I23" s="3">
-        <v>12000.00</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" t="s">
-        <v>28</v>
-      </c>
-      <c r="B24" s="3">
-        <v>0</v>
-      </c>
-      <c r="C24" s="3">
-        <v>0</v>
-      </c>
-      <c r="D24" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="E24" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="F24" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="G24" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="H24" s="3">
-        <v>0</v>
-      </c>
-      <c r="I24" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" t="s">
-        <v>29</v>
-      </c>
-      <c r="B25" s="3">
-        <v>0</v>
-      </c>
-      <c r="C25" s="3">
-        <v>0</v>
-      </c>
-      <c r="D25" s="3">
-        <v>10000.00</v>
-      </c>
-      <c r="E25" s="3">
-        <v>10000.00</v>
-      </c>
-      <c r="F25" s="3">
-        <v>10000.00</v>
-      </c>
-      <c r="G25" s="3">
-        <v>10000.00</v>
-      </c>
-      <c r="H25" s="3">
-        <v>0</v>
-      </c>
-      <c r="I25" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" t="s">
-        <v>30</v>
-      </c>
-      <c r="B26" s="3">
-        <v>0</v>
-      </c>
-      <c r="C26" s="3">
-        <v>0</v>
-      </c>
-      <c r="D26" s="3">
-        <v>3669105.60</v>
-      </c>
-      <c r="E26" s="3">
-        <v>3882225.60</v>
-      </c>
-      <c r="F26" s="3">
-        <v>3669105.60</v>
-      </c>
-      <c r="G26" s="3">
-        <v>3882225.60</v>
-      </c>
-      <c r="H26" s="3">
-        <v>0</v>
-      </c>
-      <c r="I26" s="3">
-        <v>213120.00</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="A27" t="s">
-        <v>31</v>
-      </c>
-      <c r="B27" s="3">
-        <v>0</v>
-      </c>
-      <c r="C27" s="3">
-        <v>92820.00</v>
-      </c>
-      <c r="D27" s="3">
-        <v>1021020.00</v>
-      </c>
-      <c r="E27" s="3">
-        <v>928200.00</v>
-      </c>
-      <c r="F27" s="3">
-        <v>1021020.00</v>
-      </c>
-      <c r="G27" s="3">
-        <v>1021020.00</v>
-      </c>
-      <c r="H27" s="3">
-        <v>0</v>
-      </c>
-      <c r="I27" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="A28" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="3">
-        <v>0</v>
-      </c>
-      <c r="C28" s="3">
-        <v>48064.79</v>
-      </c>
-      <c r="D28" s="3">
-        <v>524886.87</v>
-      </c>
-      <c r="E28" s="3">
-        <v>476822.08</v>
-      </c>
-      <c r="F28" s="3">
-        <v>524886.87</v>
-      </c>
-      <c r="G28" s="3">
-        <v>524886.87</v>
-      </c>
-      <c r="H28" s="3">
-        <v>0</v>
-      </c>
-      <c r="I28" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" t="s">
-        <v>33</v>
-      </c>
-      <c r="B29" s="3">
-        <v>0</v>
-      </c>
-      <c r="C29" s="3">
-        <v>319490.27</v>
-      </c>
-      <c r="D29" s="3">
-        <v>1202130.75</v>
-      </c>
-      <c r="E29" s="3">
-        <v>974675.06</v>
-      </c>
-      <c r="F29" s="3">
-        <v>1202130.75</v>
-      </c>
-      <c r="G29" s="3">
-        <v>1294165.33</v>
-      </c>
-      <c r="H29" s="3">
-        <v>0</v>
-      </c>
-      <c r="I29" s="3">
-        <v>92034.58</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="A30" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" s="3">
-        <v>0</v>
-      </c>
-      <c r="C30" s="3">
-        <v>0</v>
-      </c>
-      <c r="D30" s="3">
-        <v>503982.00</v>
-      </c>
-      <c r="E30" s="3">
-        <v>536562.00</v>
-      </c>
-      <c r="F30" s="3">
-        <v>503982.00</v>
-      </c>
-      <c r="G30" s="3">
-        <v>536562.00</v>
-      </c>
-      <c r="H30" s="3">
-        <v>0</v>
-      </c>
-      <c r="I30" s="3">
-        <v>32580.00</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ispravljeno formiranje ORIS fajla
</commit_message>
<xml_diff>
--- a/pomocna_knjiga_dobavljaca_excel.xlsx
+++ b/pomocna_knjiga_dobavljaca_excel.xlsx
@@ -14,9 +14,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="24">
-  <si>
-    <t>KNJIGA DOBAVLJAČA ZA PERIOD 07.10.2025. - 26.12.2025.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="18">
+  <si>
+    <t>KNJIGA DOBAVLJAČA ZA PERIOD 01.01.2026. - 26.02.2026.</t>
   </si>
   <si>
     <t>Početno</t>
@@ -40,52 +40,34 @@
     <t>Potražuje</t>
   </si>
   <si>
-    <t>Adeco doo</t>
-  </si>
-  <si>
-    <t>Auto-moto savez Srbije</t>
-  </si>
-  <si>
-    <t>ING - PRO DOO BEOGRAD</t>
-  </si>
-  <si>
-    <t>JKP ČISTOĆA</t>
-  </si>
-  <si>
-    <t>JKP Gradsko zelenilo</t>
+    <t>IPC INFORM.POSLOVNI CENTAR</t>
+  </si>
+  <si>
+    <t>JKP Čistoća</t>
   </si>
   <si>
     <t>JKP Informatika</t>
   </si>
   <si>
-    <t>M-S Hermes</t>
-  </si>
-  <si>
-    <t>OFFICE TREND , Beograd</t>
-  </si>
-  <si>
-    <t>Poslovni biro doo</t>
-  </si>
-  <si>
-    <t>PTT POŠTA</t>
-  </si>
-  <si>
-    <t>SAS-CS COMPANY - NOVI SAD</t>
+    <t>JKP Parking servis</t>
+  </si>
+  <si>
+    <t>NIS Gasprom</t>
   </si>
   <si>
     <t>T&amp;M GROUP SOLUTIONS doo</t>
   </si>
   <si>
-    <t>TDV FLEET SOLUTIONS</t>
-  </si>
-  <si>
-    <t>TELEKOM SRBIJA</t>
-  </si>
-  <si>
-    <t>UPRAVA ZA ZAJED.POSL.POKRAJ.ORGANA</t>
-  </si>
-  <si>
-    <t>ZOMA</t>
+    <t>TDV Fleet solutions</t>
+  </si>
+  <si>
+    <t>Telekom Srbija</t>
+  </si>
+  <si>
+    <t>Triax</t>
+  </si>
+  <si>
+    <t>Uprava za zajed.posl.pokr.organa</t>
   </si>
 </sst>
 </file>
@@ -441,14 +423,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="50.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="8" width="10" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="7" width="10" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -523,16 +505,16 @@
         <v>0</v>
       </c>
       <c r="D4" s="3">
-        <v>3456.00</v>
+        <v>57000.00</v>
       </c>
       <c r="E4" s="3">
-        <v>3456.00</v>
+        <v>57000.00</v>
       </c>
       <c r="F4" s="3">
-        <v>3456.00</v>
+        <v>57000.00</v>
       </c>
       <c r="G4" s="3">
-        <v>3456.00</v>
+        <v>57000.00</v>
       </c>
       <c r="H4" s="3">
         <v>0</v>
@@ -549,19 +531,19 @@
         <v>0</v>
       </c>
       <c r="C5" s="3">
-        <v>0</v>
+        <v>22332.29</v>
       </c>
       <c r="D5" s="3">
-        <v>28200.00</v>
+        <v>44664.58</v>
       </c>
       <c r="E5" s="3">
-        <v>28200.00</v>
+        <v>22332.29</v>
       </c>
       <c r="F5" s="3">
-        <v>28200.00</v>
+        <v>44664.58</v>
       </c>
       <c r="G5" s="3">
-        <v>28200.00</v>
+        <v>44664.58</v>
       </c>
       <c r="H5" s="3">
         <v>0</v>
@@ -578,19 +560,19 @@
         <v>0</v>
       </c>
       <c r="C6" s="3">
-        <v>0</v>
+        <v>1244.00</v>
       </c>
       <c r="D6" s="3">
-        <v>47300.00</v>
+        <v>2488.00</v>
       </c>
       <c r="E6" s="3">
-        <v>47300.00</v>
+        <v>1244.00</v>
       </c>
       <c r="F6" s="3">
-        <v>47300.00</v>
+        <v>2488.00</v>
       </c>
       <c r="G6" s="3">
-        <v>47300.00</v>
+        <v>2488.00</v>
       </c>
       <c r="H6" s="3">
         <v>0</v>
@@ -610,22 +592,22 @@
         <v>0</v>
       </c>
       <c r="D7" s="3">
-        <v>22332.29</v>
+        <v>358602.82</v>
       </c>
       <c r="E7" s="3">
-        <v>44664.58</v>
+        <v>462202.82</v>
       </c>
       <c r="F7" s="3">
-        <v>22332.29</v>
+        <v>358602.82</v>
       </c>
       <c r="G7" s="3">
-        <v>44664.58</v>
+        <v>462202.82</v>
       </c>
       <c r="H7" s="3">
         <v>0</v>
       </c>
       <c r="I7" s="3">
-        <v>22332.29</v>
+        <v>103600.00</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -639,16 +621,16 @@
         <v>0</v>
       </c>
       <c r="D8" s="3">
-        <v>75600.00</v>
+        <v>80000.00</v>
       </c>
       <c r="E8" s="3">
-        <v>75600.00</v>
+        <v>80000.00</v>
       </c>
       <c r="F8" s="3">
-        <v>75600.00</v>
+        <v>80000.00</v>
       </c>
       <c r="G8" s="3">
-        <v>75600.00</v>
+        <v>80000.00</v>
       </c>
       <c r="H8" s="3">
         <v>0</v>
@@ -665,25 +647,25 @@
         <v>0</v>
       </c>
       <c r="C9" s="3">
-        <v>0</v>
+        <v>382363.20</v>
       </c>
       <c r="D9" s="3">
-        <v>2488.00</v>
+        <v>727934.40</v>
       </c>
       <c r="E9" s="3">
-        <v>3732.00</v>
+        <v>345571.20</v>
       </c>
       <c r="F9" s="3">
-        <v>2488.00</v>
+        <v>727934.40</v>
       </c>
       <c r="G9" s="3">
-        <v>3732.00</v>
+        <v>727934.40</v>
       </c>
       <c r="H9" s="3">
         <v>0</v>
       </c>
       <c r="I9" s="3">
-        <v>1244.00</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:9">
@@ -694,19 +676,19 @@
         <v>0</v>
       </c>
       <c r="C10" s="3">
-        <v>0</v>
+        <v>92820.00</v>
       </c>
       <c r="D10" s="3">
-        <v>87463.80</v>
+        <v>185640.00</v>
       </c>
       <c r="E10" s="3">
-        <v>87463.80</v>
+        <v>92820.00</v>
       </c>
       <c r="F10" s="3">
-        <v>87463.80</v>
+        <v>185640.00</v>
       </c>
       <c r="G10" s="3">
-        <v>87463.80</v>
+        <v>185640.00</v>
       </c>
       <c r="H10" s="3">
         <v>0</v>
@@ -723,19 +705,19 @@
         <v>0</v>
       </c>
       <c r="C11" s="3">
-        <v>0</v>
+        <v>47739.37</v>
       </c>
       <c r="D11" s="3">
-        <v>54028.80</v>
+        <v>95429.53</v>
       </c>
       <c r="E11" s="3">
-        <v>54028.80</v>
+        <v>47690.16</v>
       </c>
       <c r="F11" s="3">
-        <v>54028.80</v>
+        <v>95429.53</v>
       </c>
       <c r="G11" s="3">
-        <v>54028.80</v>
+        <v>95429.53</v>
       </c>
       <c r="H11" s="3">
         <v>0</v>
@@ -755,16 +737,16 @@
         <v>0</v>
       </c>
       <c r="D12" s="3">
-        <v>4400.00</v>
+        <v>5000.00</v>
       </c>
       <c r="E12" s="3">
-        <v>4400.00</v>
+        <v>5000.00</v>
       </c>
       <c r="F12" s="3">
-        <v>4400.00</v>
+        <v>5000.00</v>
       </c>
       <c r="G12" s="3">
-        <v>4400.00</v>
+        <v>5000.00</v>
       </c>
       <c r="H12" s="3">
         <v>0</v>
@@ -781,198 +763,24 @@
         <v>0</v>
       </c>
       <c r="C13" s="3">
-        <v>0</v>
+        <v>263260.35</v>
       </c>
       <c r="D13" s="3">
-        <v>12000.00</v>
+        <v>263260.35</v>
       </c>
       <c r="E13" s="3">
-        <v>12000.00</v>
+        <v>0</v>
       </c>
       <c r="F13" s="3">
-        <v>12000.00</v>
+        <v>263260.35</v>
       </c>
       <c r="G13" s="3">
-        <v>12000.00</v>
+        <v>263260.35</v>
       </c>
       <c r="H13" s="3">
         <v>0</v>
       </c>
       <c r="I13" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="3">
-        <v>0</v>
-      </c>
-      <c r="C14" s="3">
-        <v>0</v>
-      </c>
-      <c r="D14" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="E14" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="F14" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="G14" s="3">
-        <v>239160.00</v>
-      </c>
-      <c r="H14" s="3">
-        <v>0</v>
-      </c>
-      <c r="I14" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-      <c r="B15" s="3">
-        <v>0</v>
-      </c>
-      <c r="C15" s="3">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3">
-        <v>970488.00</v>
-      </c>
-      <c r="E15" s="3">
-        <v>902696.40</v>
-      </c>
-      <c r="F15" s="3">
-        <v>970488.00</v>
-      </c>
-      <c r="G15" s="3">
-        <v>902696.40</v>
-      </c>
-      <c r="H15" s="3">
-        <v>67791.60</v>
-      </c>
-      <c r="I15" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
-      <c r="A16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B16" s="3">
-        <v>0</v>
-      </c>
-      <c r="C16" s="3">
-        <v>0</v>
-      </c>
-      <c r="D16" s="3">
-        <v>173663.22</v>
-      </c>
-      <c r="E16" s="3">
-        <v>266483.22</v>
-      </c>
-      <c r="F16" s="3">
-        <v>173663.22</v>
-      </c>
-      <c r="G16" s="3">
-        <v>266483.22</v>
-      </c>
-      <c r="H16" s="3">
-        <v>0</v>
-      </c>
-      <c r="I16" s="3">
-        <v>92820.00</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="3">
-        <v>0</v>
-      </c>
-      <c r="C17" s="3">
-        <v>0</v>
-      </c>
-      <c r="D17" s="3">
-        <v>95748.29</v>
-      </c>
-      <c r="E17" s="3">
-        <v>143932.09</v>
-      </c>
-      <c r="F17" s="3">
-        <v>95748.29</v>
-      </c>
-      <c r="G17" s="3">
-        <v>143932.09</v>
-      </c>
-      <c r="H17" s="3">
-        <v>0</v>
-      </c>
-      <c r="I17" s="3">
-        <v>48183.80</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" t="s">
-        <v>22</v>
-      </c>
-      <c r="B18" s="3">
-        <v>0</v>
-      </c>
-      <c r="C18" s="3">
-        <v>0</v>
-      </c>
-      <c r="D18" s="3">
-        <v>358355.02</v>
-      </c>
-      <c r="E18" s="3">
-        <v>183325.26</v>
-      </c>
-      <c r="F18" s="3">
-        <v>358355.02</v>
-      </c>
-      <c r="G18" s="3">
-        <v>183325.26</v>
-      </c>
-      <c r="H18" s="3">
-        <v>175029.76</v>
-      </c>
-      <c r="I18" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="3">
-        <v>0</v>
-      </c>
-      <c r="C19" s="3">
-        <v>0</v>
-      </c>
-      <c r="D19" s="3">
-        <v>244080.00</v>
-      </c>
-      <c r="E19" s="3">
-        <v>244080.00</v>
-      </c>
-      <c r="F19" s="3">
-        <v>244080.00</v>
-      </c>
-      <c r="G19" s="3">
-        <v>244080.00</v>
-      </c>
-      <c r="H19" s="3">
-        <v>0</v>
-      </c>
-      <c r="I19" s="3">
         <v>0</v>
       </c>
     </row>

</xml_diff>